<commit_message>
data(ppc): cierra semana 07 (PPC 75%) y registra metas semana 08
- index.json: semana 07 cierre -> cierres/semana-07.json; alta semana 08 (29 jun - 5 jul, abierta)
- Acta de cierre y JSON de cierre de la semana 07
- Excel de metas de la semana 08 (16 compromisos)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ppc/metas/semana-07.xlsx
+++ b/data/ppc/metas/semana-07.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/06. ALTOZANO - TABLERO GENERAL/data/ppc/metas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="8_{630896EA-F834-475B-A060-53197EEC23A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D552B9A9-531F-4A77-9D50-CDE4ACA55A35}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{630896EA-F834-475B-A060-53197EEC23A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B669DBD-EDEF-4C63-81F3-75264849EC73}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Metas Semana 05" sheetId="1" r:id="rId1"/>
+    <sheet name="Metas Semana 07" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -187,9 +187,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -634,7 +631,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="3" t="s">

</xml_diff>